<commit_message>
Added time relted artifacts
</commit_message>
<xml_diff>
--- a/314e-ig/output/StructureDefinition-annotation-314e.xlsx
+++ b/314e-ig/output/StructureDefinition-annotation-314e.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="130">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-16T13:10:22+05:30</t>
+    <t>2026-05-16T16:45:26+05:30</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -375,20 +375,36 @@
     <t>Organization is used when there's no need for specific attribution as to who made the comment.</t>
   </si>
   <si>
+    <t xml:space="preserve">type:$this}
+</t>
+  </si>
+  <si>
     <t>Act.participant[typeCode=AUT].role</t>
   </si>
   <si>
+    <t>Annotation.author[x]:authorReference</t>
+  </si>
+  <si>
+    <t>authorReference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference(Practitioner|Patient|RelatedPerson|Organization) {http://314e.com/fhir/StructureDefinition/reference-314e}
+</t>
+  </si>
+  <si>
     <t>Annotation.time</t>
   </si>
   <si>
-    <t xml:space="preserve">dateTime
+    <t xml:space="preserve">dateTime {http://314e.com/fhir/ig/StructureDefinition/datetime-314e}
 </t>
   </si>
   <si>
-    <t>When the annotation was made</t>
-  </si>
-  <si>
-    <t>Indicates when this particular annotation was made.</t>
+    <t>Annotation time in UTC with precision support</t>
+  </si>
+  <si>
+    <t>Date/time when the annotation was made.
+All timestamps SHALL be represented in UTC.
+Precision and approximation extensions may be used.</t>
   </si>
   <si>
     <t>Act.effectiveTime</t>
@@ -711,12 +727,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AL8"/>
+  <dimension ref="A1:AL9"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="28.1640625" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="32.046875" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="18.296875" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="10.26953125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="3" max="3" width="14.49609375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="11.10546875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.29296875" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.21484375" customWidth="true" bestFit="true"/>
@@ -724,7 +740,7 @@
     <col min="8" max="8" width="13.1171875" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="10.75390625" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="69.7890625" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="98.0859375" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -1374,16 +1390,14 @@
         <v>20</v>
       </c>
       <c r="AB6" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AC6" t="s" s="2">
-        <v>20</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="AC6" s="2"/>
       <c r="AD6" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AE6" t="s" s="2">
-        <v>20</v>
+        <v>101</v>
       </c>
       <c r="AF6" t="s" s="2">
         <v>109</v>
@@ -1404,17 +1418,19 @@
         <v>84</v>
       </c>
       <c r="AL6" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="C7" s="2"/>
+        <v>109</v>
+      </c>
+      <c r="C7" t="s" s="2">
+        <v>118</v>
+      </c>
       <c r="D7" t="s" s="2">
         <v>20</v>
       </c>
@@ -1435,15 +1451,17 @@
         <v>110</v>
       </c>
       <c r="K7" t="s" s="2">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L7" t="s" s="2">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="M7" t="s" s="2">
-        <v>119</v>
-      </c>
-      <c r="N7" s="2"/>
+        <v>113</v>
+      </c>
+      <c r="N7" t="s" s="2">
+        <v>114</v>
+      </c>
       <c r="O7" s="2"/>
       <c r="P7" t="s" s="2">
         <v>20</v>
@@ -1492,7 +1510,7 @@
         <v>20</v>
       </c>
       <c r="AF7" t="s" s="2">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="AG7" t="s" s="2">
         <v>76</v>
@@ -1510,15 +1528,15 @@
         <v>84</v>
       </c>
       <c r="AL7" t="s" s="2">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" t="s" s="2">
@@ -1526,7 +1544,7 @@
       </c>
       <c r="E8" s="2"/>
       <c r="F8" t="s" s="2">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="G8" t="s" s="2">
         <v>87</v>
@@ -1541,13 +1559,13 @@
         <v>110</v>
       </c>
       <c r="K8" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="L8" t="s" s="2">
         <v>122</v>
       </c>
-      <c r="L8" t="s" s="2">
+      <c r="M8" t="s" s="2">
         <v>123</v>
-      </c>
-      <c r="M8" t="s" s="2">
-        <v>124</v>
       </c>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
@@ -1598,10 +1616,10 @@
         <v>20</v>
       </c>
       <c r="AF8" t="s" s="2">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="AG8" t="s" s="2">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="AH8" t="s" s="2">
         <v>87</v>
@@ -1616,7 +1634,113 @@
         <v>84</v>
       </c>
       <c r="AL8" t="s" s="2">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="2">
         <v>125</v>
+      </c>
+      <c r="B9" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="C9" s="2"/>
+      <c r="D9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="E9" s="2"/>
+      <c r="F9" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="G9" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="I9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="J9" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="K9" t="s" s="2">
+        <v>126</v>
+      </c>
+      <c r="L9" t="s" s="2">
+        <v>127</v>
+      </c>
+      <c r="M9" t="s" s="2">
+        <v>128</v>
+      </c>
+      <c r="N9" s="2"/>
+      <c r="O9" s="2"/>
+      <c r="P9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Q9" s="2"/>
+      <c r="R9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="S9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="T9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="U9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="V9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="W9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="X9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Y9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Z9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AA9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AB9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AC9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AD9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AE9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AF9" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="AG9" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AH9" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AJ9" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AK9" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AL9" t="s" s="2">
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>